<commit_message>
docs(reports): Consolidado oficial PAS actualizado con resultado real 10/19 (v7.5)
</commit_message>
<xml_diff>
--- a/ReportesTrades/PokerDeAses/PAS_10192026.xlsx
+++ b/ReportesTrades/PokerDeAses/PAS_10192026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="72">
   <si>
     <t>$162.50</t>
   </si>
@@ -37,9 +37,6 @@
     <t>Profit</t>
   </si>
   <si>
-    <t>$150.00</t>
-  </si>
-  <si>
     <t>7771.75</t>
   </si>
   <si>
@@ -70,9 +67,6 @@
     <t>Qty</t>
   </si>
   <si>
-    <t>Z1_Mono_Tp</t>
-  </si>
-  <si>
     <t>$237.50</t>
   </si>
   <si>
@@ -100,9 +94,6 @@
     <t>Cascada_Mono_SL</t>
   </si>
   <si>
-    <t>$95.64</t>
-  </si>
-  <si>
     <t>$254.36</t>
   </si>
   <si>
@@ -178,12 +169,6 @@
     <t>Short</t>
   </si>
   <si>
-    <t>7749.25</t>
-  </si>
-  <si>
-    <t>($434.88)</t>
-  </si>
-  <si>
     <t>$141.86</t>
   </si>
   <si>
@@ -226,9 +211,6 @@
     <t>Exit price</t>
   </si>
   <si>
-    <t>$54.36</t>
-  </si>
-  <si>
     <t>Cascada50_Long</t>
   </si>
   <si>
@@ -248,9 +230,6 @@
   </si>
   <si>
     <t>$13.08</t>
-  </si>
-  <si>
-    <t>7751.25</t>
   </si>
 </sst>
 </file>
@@ -587,82 +566,85 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J7"/>
+  <dimension ref="A1:J6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="23" width="11" customWidth="1"/>
+    <col min="1" max="10" width="10.28515625" customWidth="1"/>
+    <col min="11" max="11" width="15" customWidth="1"/>
+    <col min="12" max="12" width="22.5703125" customWidth="1"/>
+    <col min="13" max="23" width="10.28515625" customWidth="1"/>
     <col min="24" max="16384" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" ht="19.5" customHeight="1">
       <c r="A1" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="B1" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="C1" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="D1" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="E1" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="F1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G1" t="s">
         <v>4</v>
       </c>
       <c r="H1" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="I1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="J1" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="K1" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="L1" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="M1" t="s">
         <v>6</v>
       </c>
       <c r="N1" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="O1" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="P1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="Q1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="R1" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="S1" t="s">
         <v>2</v>
       </c>
       <c r="T1" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="U1" t="s">
+        <v>42</v>
+      </c>
+      <c r="V1" t="s">
+        <v>31</v>
+      </c>
+      <c r="W1" t="s">
         <v>45</v>
-      </c>
-      <c r="V1" t="s">
-        <v>34</v>
-      </c>
-      <c r="W1" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="2" ht="15.75" customHeight="1">
@@ -670,25 +652,25 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C2" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="D2" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="E2" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="F2" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="G2" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="H2" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="I2" s="1">
         <v>46314.4257407407</v>
@@ -697,40 +679,40 @@
         <v>46314.4264351852</v>
       </c>
       <c r="K2" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="L2" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="M2" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="N2" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="O2" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="P2" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="Q2" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="R2" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="S2" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="T2" t="s">
         <v>1</v>
       </c>
       <c r="U2" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="V2" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="W2">
         <v>9</v>
@@ -741,25 +723,25 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C3" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="D3" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="E3" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="F3" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="G3" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="H3" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="I3" s="1">
         <v>46314.4411458333</v>
@@ -768,37 +750,37 @@
         <v>46314.4417361111</v>
       </c>
       <c r="K3" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="L3" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="M3" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="N3" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="O3" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="P3" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="Q3" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="R3" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="S3" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="T3" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="U3" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="V3" t="s">
         <v>3</v>
@@ -812,25 +794,25 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C4" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="D4" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="E4" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="F4" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="G4" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="H4" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="I4" s="1">
         <v>46314.458599537</v>
@@ -839,40 +821,40 @@
         <v>46314.4627546296</v>
       </c>
       <c r="K4" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="L4" t="s">
+        <v>18</v>
+      </c>
+      <c r="M4" t="s">
+        <v>66</v>
+      </c>
+      <c r="N4" t="s">
+        <v>40</v>
+      </c>
+      <c r="O4" t="s">
+        <v>53</v>
+      </c>
+      <c r="P4" t="s">
+        <v>70</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>70</v>
+      </c>
+      <c r="R4" t="s">
+        <v>70</v>
+      </c>
+      <c r="S4" t="s">
+        <v>70</v>
+      </c>
+      <c r="T4" t="s">
+        <v>17</v>
+      </c>
+      <c r="U4" t="s">
         <v>20</v>
       </c>
-      <c r="M4" t="s">
-        <v>72</v>
-      </c>
-      <c r="N4" t="s">
-        <v>43</v>
-      </c>
-      <c r="O4" t="s">
-        <v>58</v>
-      </c>
-      <c r="P4" t="s">
-        <v>76</v>
-      </c>
-      <c r="Q4" t="s">
-        <v>76</v>
-      </c>
-      <c r="R4" t="s">
-        <v>76</v>
-      </c>
-      <c r="S4" t="s">
-        <v>76</v>
-      </c>
-      <c r="T4" t="s">
-        <v>19</v>
-      </c>
-      <c r="U4" t="s">
-        <v>22</v>
-      </c>
       <c r="V4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="W4">
         <v>27</v>
@@ -883,25 +865,25 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C5" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="D5" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="E5" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="F5" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="G5" t="s">
         <v>5</v>
       </c>
       <c r="H5" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="I5" s="1">
         <v>46314.4778472222</v>
@@ -910,31 +892,31 @@
         <v>46314.4788194444</v>
       </c>
       <c r="K5" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="L5" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="M5" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="N5" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="O5" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="P5" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="Q5" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="R5" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="S5" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="T5" t="s">
         <v>0</v>
@@ -943,7 +925,7 @@
         <v>1</v>
       </c>
       <c r="V5" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="W5">
         <v>9</v>
@@ -954,25 +936,25 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C6" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="D6" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="E6" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="F6" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="G6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H6" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="I6" s="1">
         <v>46314.4838310185</v>
@@ -981,114 +963,43 @@
         <v>46314.48625</v>
       </c>
       <c r="K6" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="L6" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="M6" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="N6" t="s">
+        <v>12</v>
+      </c>
+      <c r="O6" t="s">
+        <v>53</v>
+      </c>
+      <c r="P6" t="s">
+        <v>70</v>
+      </c>
+      <c r="Q6" t="s">
+        <v>70</v>
+      </c>
+      <c r="R6" t="s">
+        <v>70</v>
+      </c>
+      <c r="S6" t="s">
+        <v>70</v>
+      </c>
+      <c r="T6" t="s">
+        <v>20</v>
+      </c>
+      <c r="U6" t="s">
         <v>13</v>
       </c>
-      <c r="O6" t="s">
-        <v>58</v>
-      </c>
-      <c r="P6" t="s">
-        <v>76</v>
-      </c>
-      <c r="Q6" t="s">
-        <v>76</v>
-      </c>
-      <c r="R6" t="s">
-        <v>76</v>
-      </c>
-      <c r="S6" t="s">
-        <v>76</v>
-      </c>
-      <c r="T6" t="s">
-        <v>22</v>
-      </c>
-      <c r="U6" t="s">
-        <v>14</v>
-      </c>
       <c r="V6" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="W6">
         <v>13</v>
-      </c>
-    </row>
-    <row r="7" ht="15.75" customHeight="1">
-      <c r="A7">
-        <v>6</v>
-      </c>
-      <c r="B7" t="s">
-        <v>11</v>
-      </c>
-      <c r="C7" t="s">
-        <v>30</v>
-      </c>
-      <c r="D7" t="s">
-        <v>67</v>
-      </c>
-      <c r="E7" t="s">
-        <v>53</v>
-      </c>
-      <c r="F7" t="s">
-        <v>46</v>
-      </c>
-      <c r="G7" t="s">
-        <v>78</v>
-      </c>
-      <c r="H7" t="s">
-        <v>54</v>
-      </c>
-      <c r="I7" s="1">
-        <v>46314.5027314815</v>
-      </c>
-      <c r="J7" s="1">
-        <v>46314.5044907407</v>
-      </c>
-      <c r="K7" t="s">
-        <v>42</v>
-      </c>
-      <c r="L7" t="s">
-        <v>18</v>
-      </c>
-      <c r="M7" t="s">
-        <v>28</v>
-      </c>
-      <c r="N7" t="s">
-        <v>55</v>
-      </c>
-      <c r="O7" t="s">
-        <v>58</v>
-      </c>
-      <c r="P7" t="s">
-        <v>76</v>
-      </c>
-      <c r="Q7" t="s">
-        <v>76</v>
-      </c>
-      <c r="R7" t="s">
-        <v>76</v>
-      </c>
-      <c r="S7" t="s">
-        <v>76</v>
-      </c>
-      <c r="T7" t="s">
-        <v>0</v>
-      </c>
-      <c r="U7" t="s">
-        <v>7</v>
-      </c>
-      <c r="V7" t="s">
-        <v>70</v>
-      </c>
-      <c r="W7">
-        <v>15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>